<commit_message>
Endpoint liviano de respuestas por codigo, modulo Acceso a Clientes, y fix de solicitudes duplicadas
Nuevo GET /solicitudes/:id/respuestas-por-codigo (formulario-renderizable.service.ts)
para resolver 2-4 preguntas puntuales sin renderizar el formulario completo -
usado por el bloque "Solicita cupo de credito" de las pantallas de gestion,
que antes tardaba varios segundos por depender del render completo (~85-100
preguntas). Migracion para el submodulo "Acceso a Clientes" bajo
Parametrizacion > Clientes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentos Cartonera/PORTAL Y PQRS.xlsx
+++ b/Documentos Cartonera/PORTAL Y PQRS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\Cartonera\PROYECTO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DAVID\CN\B_PortalClientes\Documentos Cartonera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6CCD3B0-4137-4DA5-978B-A8845C398DB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3BD6535-88BE-4697-87CB-BB92D8A1C18A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{8D8B2D89-AFE5-42E6-B2E1-0EDE2B1A6320}"/>
+    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10060" activeTab="3" xr2:uid="{8D8B2D89-AFE5-42E6-B2E1-0EDE2B1A6320}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -830,13 +830,57 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>627524</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>40533</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7238430E-3E74-BA84-BC8D-9135F7999DB8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6096000" y="184150"/>
+          <a:ext cx="9009524" cy="5933333"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -874,7 +918,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -980,7 +1024,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1122,7 +1166,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1131,15 +1175,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60830835-8A6B-40F8-9D8D-547F84799DB6}">
   <dimension ref="A2:E13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" customWidth="1"/>
-    <col min="3" max="3" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.90625" customWidth="1"/>
+    <col min="3" max="3" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
@@ -1150,7 +1194,7 @@
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1161,7 +1205,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1192,7 +1236,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>6</v>
       </c>
@@ -1203,7 +1247,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>9</v>
       </c>
@@ -1214,7 +1258,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>11</v>
       </c>
@@ -1225,7 +1269,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
         <v>15</v>
       </c>
@@ -1236,7 +1280,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>16</v>
       </c>
@@ -1247,7 +1291,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>17</v>
       </c>
@@ -1258,7 +1302,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1275,7 +1319,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1304,19 +1348,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D67EAD8A-91A3-4375-BD54-D978BD967765}">
   <dimension ref="A1:H82"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>40</v>
       </c>
@@ -1342,7 +1386,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1368,7 +1412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1394,7 +1438,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1420,7 +1464,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1446,7 +1490,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
@@ -1472,7 +1516,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1498,7 +1542,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1524,7 +1568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1550,7 +1594,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2</v>
       </c>
@@ -1576,7 +1620,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1602,7 +1646,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>3</v>
       </c>
@@ -1628,7 +1672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>3</v>
       </c>
@@ -1654,7 +1698,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>3</v>
       </c>
@@ -1680,7 +1724,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>3</v>
       </c>
@@ -1706,7 +1750,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>3</v>
       </c>
@@ -1732,7 +1776,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>3</v>
       </c>
@@ -1758,7 +1802,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>4</v>
       </c>
@@ -1784,7 +1828,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>4</v>
       </c>
@@ -1810,7 +1854,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>4</v>
       </c>
@@ -1836,7 +1880,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>4</v>
       </c>
@@ -1862,7 +1906,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>4</v>
       </c>
@@ -1888,7 +1932,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>5</v>
       </c>
@@ -1914,7 +1958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>5</v>
       </c>
@@ -1940,7 +1984,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>5</v>
       </c>
@@ -1966,7 +2010,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>5</v>
       </c>
@@ -1992,7 +2036,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -2006,7 +2050,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>1</v>
       </c>
@@ -2020,7 +2064,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2</v>
       </c>
@@ -2034,7 +2078,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>3</v>
       </c>
@@ -2048,7 +2092,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>4</v>
       </c>
@@ -2062,7 +2106,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>5</v>
       </c>
@@ -2076,7 +2120,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>6</v>
       </c>
@@ -2090,7 +2134,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>7</v>
       </c>
@@ -2104,7 +2148,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>8</v>
       </c>
@@ -2118,7 +2162,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>9</v>
       </c>
@@ -2132,7 +2176,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>10</v>
       </c>
@@ -2146,7 +2190,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>11</v>
       </c>
@@ -2160,7 +2204,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>12</v>
       </c>
@@ -2174,7 +2218,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>13</v>
       </c>
@@ -2188,7 +2232,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>14</v>
       </c>
@@ -2202,7 +2246,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>15</v>
       </c>
@@ -2216,7 +2260,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>16</v>
       </c>
@@ -2230,7 +2274,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>17</v>
       </c>
@@ -2244,7 +2288,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>18</v>
       </c>
@@ -2258,7 +2302,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>19</v>
       </c>
@@ -2272,7 +2316,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>20</v>
       </c>
@@ -2286,7 +2330,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>21</v>
       </c>
@@ -2300,7 +2344,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>22</v>
       </c>
@@ -2314,7 +2358,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>23</v>
       </c>
@@ -2328,7 +2372,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>24</v>
       </c>
@@ -2342,7 +2386,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>25</v>
       </c>
@@ -2356,12 +2400,12 @@
         <v>166</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>59</v>
       </c>
@@ -2369,7 +2413,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>169</v>
       </c>
@@ -2377,7 +2421,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>171</v>
       </c>
@@ -2385,7 +2429,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>56</v>
       </c>
@@ -2393,7 +2437,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>174</v>
       </c>
@@ -2401,7 +2445,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>176</v>
       </c>
@@ -2409,7 +2453,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>178</v>
       </c>
@@ -2417,7 +2461,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>180</v>
       </c>
@@ -2425,7 +2469,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>182</v>
       </c>
@@ -2433,7 +2477,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>184</v>
       </c>
@@ -2441,62 +2485,62 @@
         <v>185</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>53</v>
       </c>
@@ -2510,18 +2554,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{366F6ECE-C492-427B-A488-1207C48EDF72}">
   <dimension ref="B1:J27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="41.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="41.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="3:10" x14ac:dyDescent="0.35">
       <c r="D1" t="s">
         <v>197</v>
       </c>
@@ -2541,7 +2585,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="2" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
         <v>201</v>
       </c>
@@ -2549,73 +2593,73 @@
         <v>202</v>
       </c>
     </row>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="7" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="9" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="11" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="14" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C14" s="1" t="s">
         <v>206</v>
       </c>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C16" t="s">
         <v>208</v>
       </c>
@@ -2623,39 +2667,39 @@
         <v>209</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C18" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C19" t="s">
         <v>212</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C20" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C21" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C22" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>220</v>
       </c>
@@ -2663,22 +2707,22 @@
         <v>219</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C24" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C25" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C26" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C27" t="s">
         <v>224</v>
       </c>
@@ -2692,7 +2736,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89FE3A69-FA62-4A45-A6CD-E63B1F1C9C08}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>